<commit_message>
Update XLSX parser to extract concrete material properties from IFC reports
Key features implemented:
- Modified xlsx_parser.py to identify load-bearing concrete elements (walls, slabs, columns, footings, beams, members)
- Added extraction of concrete material properties: class (grade), frost resistance, water permeability
- Updated parsing logic to handle multiple report structures and locate material property columns
- Enhanced material aggregation to include concrete characteristics in the summary
- Modified output Excel format to include concrete grade, frost resistance, and water resistance columns
- Updated JSON output schema to include the new material property fields
- Improved material detection fallback logic using element names and object types

The updated parser now correctly processes both specified IFC report formats and generates comprehensive material summaries including essential concrete properties for structural elements.
</commit_message>
<xml_diff>
--- a/uploads/384edf8f-ae4d-4ba9-9632-790977e6a93a/materials_summary.xlsx
+++ b/uploads/384edf8f-ae4d-4ba9-9632-790977e6a93a/materials_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Сводка по элементам" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка по элементам" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,15 +433,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,15 +465,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Класс бетона</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Морозостойкость</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Водонепроницаемость</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Количество, шт</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Объем, м³</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Площадь, м²</t>
         </is>
@@ -492,13 +510,28 @@
           <t>Железобетон B25</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>F100</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>12667.114</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="I2" s="2" t="n">
         <v>152394440</v>
       </c>
     </row>
@@ -518,13 +551,28 @@
           <t>Железобетон B30</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>F150</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>2778.396</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="I3" s="2" t="n">
         <v>70254484.55</v>
       </c>
     </row>
@@ -544,13 +592,28 @@
           <t>Сталь</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>164.1</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="I4" s="2" t="n">
         <v>45318532.299</v>
       </c>
     </row>
@@ -570,15 +633,30 @@
           <t>Железобетон B30</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>F150</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -600,13 +678,28 @@
           <t>М</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>1014938.63</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="I6" s="2" t="n">
         <v>1735925.197</v>
       </c>
     </row>
@@ -626,13 +719,28 @@
           <t>Сталь</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>0.066</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -654,13 +762,28 @@
           <t>Железобетон</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>54399.948</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -682,13 +805,28 @@
           <t>Сборный железобетон</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>4338.062</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -710,15 +848,30 @@
           <t>Железобетон</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -740,15 +893,30 @@
           <t>Железобетон В30</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>В30</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -770,13 +938,28 @@
           <t>Железобетон B25</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>F100</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>185</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>3152015.753</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="I12" s="2" t="n">
         <v>33499.008</v>
       </c>
     </row>
@@ -796,13 +979,28 @@
           <t>Железобетон B30</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>F150</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>3204423.625</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="I13" s="2" t="n">
         <v>15373.627</v>
       </c>
     </row>
@@ -822,13 +1020,28 @@
           <t>ПОД</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>8807.267</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="I14" s="2" t="n">
         <v>8279.956</v>
       </c>
     </row>
@@ -848,13 +1061,28 @@
           <t>Экструдированный пенополистирол</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>470.273</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="I15" s="2" t="n">
         <v>359.025</v>
       </c>
     </row>
@@ -874,15 +1102,30 @@
           <t>Не указан</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>103</v>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -904,15 +1147,30 @@
           <t>Не указан</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>868</v>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -934,15 +1192,30 @@
           <t>Не указан</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -964,15 +1237,30 @@
           <t>Не указан</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>367</v>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -994,13 +1282,28 @@
           <t>Железобетон B25</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>B25</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>F100</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
         <v>1468</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>2572814.24</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="I20" s="2" t="n">
         <v>24800.867</v>
       </c>
     </row>
@@ -1020,13 +1323,28 @@
           <t>Железобетон B30</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n">
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>F150</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
         <v>293</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>1338410.945</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="I21" s="2" t="n">
         <v>10907.351</v>
       </c>
     </row>
@@ -1046,13 +1364,28 @@
           <t>Не указан</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>94</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="H22" s="2" t="n">
         <v>3.541</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="I22" s="2" t="n">
         <v>321000</v>
       </c>
     </row>

</xml_diff>